<commit_message>
Final server portability hardening + VM README + verified clean venv run
</commit_message>
<xml_diff>
--- a/Parsed_PO_Lines.xlsx
+++ b/Parsed_PO_Lines.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,50 +466,35 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>ship_to</t>
+          <t>customer_product_no</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>customer_product_no</t>
+          <t>te_part_number</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>te_part_number</t>
+          <t>manufacturer_part_no</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>manufacturer_part_no</t>
+          <t>description</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>quantity</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>quantity</t>
+          <t>uom</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>uom</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>price</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>line_value</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>delivery_date</t>
         </is>
@@ -518,26 +503,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1227-2025 - TE Connect.PDF</t>
+          <t>__B01631255_080318 (1) (1) Neways Riesa - Copy.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1227/2025</t>
+          <t>11B01631255</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>01.09.2025</t>
+          <t>08.12.2025</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Boario Impianti S.r.l.</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+          <t>Neways Electronics Riesa GmbH</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Frau Bröcher</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>TE Connectivity Solutions GmbH Bestelldatum : 08.12.2025 Muehlenstraße 26 Lieferanten-Nr. : 76001 CH-8200 Schaffhausen</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>1</t>
@@ -545,68 +538,71 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>XX</t>
+          <t>VA.NER0015e</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1SET411103R0000</t>
+          <t>494996-E</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>1SET411103R0000</t>
+          <t>D:ERN 494996</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1SET411103R0000</t>
+          <t>STV 2x13pol ger RM1,27</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>CANALINA DI CABLAGGIO HALOGEN FREE 25x60</t>
-        </is>
-      </c>
-      <c r="M2" t="n">
-        <v>30</v>
+          <t>5024</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Mt</t>
-        </is>
-      </c>
-      <c r="O2" t="n">
-        <v>9.18817</v>
-      </c>
-      <c r="P2" t="n">
-        <v>275.65</v>
-      </c>
-      <c r="Q2" t="inlineStr"/>
+          <t>Not found</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1227-2025 - TE Connect.PDF</t>
+          <t>__B01631255_080318 (1) (1) Neways Riesa - Copy.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1227/2025</t>
+          <t>11B01631255</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>01.09.2025</t>
+          <t>08.12.2025</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Boario Impianti S.r.l.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+          <t>Neways Electronics Riesa GmbH</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Frau Bröcher</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>TE Connectivity Solutions GmbH Bestelldatum : 08.12.2025 Muehlenstraße 26 Lieferanten-Nr. : 76001 CH-8200 Schaffhausen</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>2</t>
@@ -614,320 +610,39 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>XX</t>
+          <t>VA.NER0015e</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>1SET411105R0000</t>
+          <t>494996-E</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>1SET411105R0000</t>
+          <t>D:ERN 494996</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1SET411105R0000</t>
+          <t>STV 2x13pol ger RM1,27</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>CANALINA DI CABLAGGIO HALOGEN FREE 40x60</t>
-        </is>
-      </c>
-      <c r="M3" t="n">
-        <v>36</v>
+          <t>5024</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Mt</t>
-        </is>
-      </c>
-      <c r="O3" t="n">
-        <v>10.85876</v>
-      </c>
-      <c r="P3" t="n">
-        <v>390.92</v>
-      </c>
-      <c r="Q3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1227-2025 - TE Connect.PDF</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>1227/2025</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>01.09.2025</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Boario Impianti S.r.l.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>XX</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>1SET411108R0000</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>1SET411108R0000</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>1SET411108R0000</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>CANALINA DI CABLAGGIO HALOGEN FREE 60x60</t>
-        </is>
-      </c>
-      <c r="M4" t="n">
-        <v>24</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Mt</t>
-        </is>
-      </c>
-      <c r="O4" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="P4" t="n">
-        <v>340.8</v>
-      </c>
-      <c r="Q4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1227-2025 - TE Connect.PDF</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>1227/2025</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>01.09.2025</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Boario Impianti S.r.l.</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>XX</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>1SET411106R0000</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>1SET411106R0000</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>1SET411106R0000</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>CANALINA DI CABLAGGIO HALOGEN FREE 40x80</t>
-        </is>
-      </c>
-      <c r="M5" t="n">
-        <v>20</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Mt</t>
-        </is>
-      </c>
-      <c r="O5" t="n">
-        <v>13.27</v>
-      </c>
-      <c r="P5" t="n">
-        <v>265.4</v>
-      </c>
-      <c r="Q5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1227-2025 - TE Connect.PDF</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>1227/2025</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>01.09.2025</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Boario Impianti S.r.l.</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>XX</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>1SET411109R0000</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>1SET411109R0000</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>1SET411109R0000</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>CANALINA DI CABLAGGIO HALOGEN FREE 60x80</t>
-        </is>
-      </c>
-      <c r="M6" t="n">
-        <v>24</v>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Mt</t>
-        </is>
-      </c>
-      <c r="O6" t="n">
-        <v>16.28</v>
-      </c>
-      <c r="P6" t="n">
-        <v>390.72</v>
-      </c>
-      <c r="Q6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1227-2025 - TE Connect.PDF</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>1227/2025</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>01.09.2025</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Boario Impianti S.r.l.</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>XX</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>1SET411111R0000</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>1SET411111R0000</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>1SET411111R0000</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>CANALINA DI CABLAGGIO HALOGEN FREE 80x80</t>
-        </is>
-      </c>
-      <c r="M7" t="n">
-        <v>10</v>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Mt</t>
-        </is>
-      </c>
-      <c r="O7" t="n">
-        <v>19.77</v>
-      </c>
-      <c r="P7" t="n">
-        <v>197.7</v>
-      </c>
-      <c r="Q7" t="inlineStr"/>
+          <t>15.06.2026</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>